<commit_message>
Agregar notificación a responsables y listado de equipos sin responsable
</commit_message>
<xml_diff>
--- a/ejemplos/plantilla_vulnerabilidades.xlsx
+++ b/ejemplos/plantilla_vulnerabilidades.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vulnerabilidades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Responsables" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,7 +485,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -594,21 +631,50 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>La app lee solo la PRIMERA hoja. Esta hoja de instrucciones va segunda.</t>
+          <t>La app lee la PRIMERA hoja (vulnerabilidades) y, si existe, la hoja 'Responsables'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Hoja Responsables</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Una fila por equipo: Activo (igual que en la primera hoja), Responsable y Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Responsable / Email</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>También se pueden poner como columnas en la primera hoja; tienen prioridad sobre la hoja Responsables</t>
         </is>
       </c>
     </row>

</xml_diff>